<commit_message>
chore: run 2026-07-08 10:57 — histórico, dashboard e Excel atualizados
</commit_message>
<xml_diff>
--- a/logs/Consolidado_08_07_2026.xlsx
+++ b/logs/Consolidado_08_07_2026.xlsx
@@ -657,10 +657,10 @@
         <v>150</v>
       </c>
       <c r="C2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
         <v>3</v>
@@ -695,7 +695,7 @@
         <v>75</v>
       </c>
       <c r="C4" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
@@ -714,7 +714,7 @@
         <v>68</v>
       </c>
       <c r="C5" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
@@ -733,7 +733,7 @@
         <v>48</v>
       </c>
       <c r="C6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
@@ -752,10 +752,10 @@
         <v>101</v>
       </c>
       <c r="C7" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="D7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E7" t="n">
         <v>23</v>
@@ -3055,38 +3055,38 @@
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="7" t="inlineStr">
+      <c r="A61" s="3" t="inlineStr">
         <is>
           <t>A-Derma</t>
         </is>
       </c>
-      <c r="B61" s="7" t="inlineStr">
+      <c r="B61" s="3" t="inlineStr">
         <is>
           <t>Exomega Control Emolient Shower Oil
 Óleo Banho Calmante Comichão da Pele Atópica</t>
         </is>
       </c>
-      <c r="C61" s="7" t="inlineStr">
+      <c r="C61" s="3" t="inlineStr">
         <is>
           <t>1000 ml</t>
         </is>
       </c>
-      <c r="D61" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="E61" s="7" t="inlineStr">
+      <c r="D61" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E61" s="3" t="inlineStr">
         <is>
           <t>8605683</t>
         </is>
       </c>
-      <c r="F61" s="7" t="inlineStr">
+      <c r="F61" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
       </c>
-      <c r="G61" s="7" t="inlineStr">
+      <c r="G61" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/exomega-control-emolient-shower-oil-452817.html</t>
         </is>
@@ -8518,38 +8518,38 @@
       </c>
     </row>
     <row r="208">
-      <c r="A208" s="7" t="inlineStr">
+      <c r="A208" s="5" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="B208" s="7" t="inlineStr">
+      <c r="B208" s="5" t="inlineStr">
         <is>
           <t>Thermal Spring Water Sensitive Skin
 Água Termal Spray Calmante Instantâneo</t>
         </is>
       </c>
-      <c r="C208" s="7" t="inlineStr">
+      <c r="C208" s="5" t="inlineStr">
         <is>
           <t>50 ml</t>
         </is>
       </c>
-      <c r="D208" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="E208" s="7" t="inlineStr">
+      <c r="D208" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E208" s="5" t="inlineStr">
         <is>
           <t>3000998</t>
         </is>
       </c>
-      <c r="F208" s="7" t="inlineStr">
+      <c r="F208" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
       </c>
-      <c r="G208" s="7" t="inlineStr">
+      <c r="G208" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/thermal-spring-water-sensitive-skin-431510.html</t>
         </is>
@@ -14654,38 +14654,38 @@
       </c>
     </row>
     <row r="373">
-      <c r="A373" s="7" t="inlineStr">
+      <c r="A373" s="3" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="B373" s="7" t="inlineStr">
+      <c r="B373" s="3" t="inlineStr">
         <is>
           <t>Mango Nourishing Shampoo
 Champô Manga Nutritivo para Cabelo Seco</t>
         </is>
       </c>
-      <c r="C373" s="7" t="inlineStr">
+      <c r="C373" s="3" t="inlineStr">
         <is>
           <t>100 ml</t>
         </is>
       </c>
-      <c r="D373" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="E373" s="7" t="inlineStr">
+      <c r="D373" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E373" s="3" t="inlineStr">
         <is>
           <t>6128309</t>
         </is>
       </c>
-      <c r="F373" s="7" t="inlineStr">
+      <c r="F373" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
       </c>
-      <c r="G373" s="7" t="inlineStr">
+      <c r="G373" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/mango-nourishing-shampoo-344278.html</t>
         </is>
@@ -15485,38 +15485,38 @@
       </c>
     </row>
     <row r="395">
-      <c r="A395" s="7" t="inlineStr">
+      <c r="A395" s="3" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="B395" s="7" t="inlineStr">
+      <c r="B395" s="3" t="inlineStr">
         <is>
           <t>Prickly Pear 72h Hydration &amp; Shine Shampoo
 Champô Figo da Índia Hidratante Cabelo Baço</t>
         </is>
       </c>
-      <c r="C395" s="7" t="inlineStr">
+      <c r="C395" s="3" t="inlineStr">
         <is>
           <t>400 ml</t>
         </is>
       </c>
-      <c r="D395" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="E395" s="7" t="inlineStr">
+      <c r="D395" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E395" s="3" t="inlineStr">
         <is>
           <t>8067439</t>
         </is>
       </c>
-      <c r="F395" s="7" t="inlineStr">
+      <c r="F395" s="3" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
       </c>
-      <c r="G395" s="7" t="inlineStr">
+      <c r="G395" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/prickly-pear-72h-hydration-and-shine-shampoo-355576.html</t>
         </is>
@@ -15820,38 +15820,38 @@
       </c>
     </row>
     <row r="404">
-      <c r="A404" s="7" t="inlineStr">
+      <c r="A404" s="3" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="B404" s="7" t="inlineStr">
+      <c r="B404" s="3" t="inlineStr">
         <is>
           <t>Quinine Strengthening Thinning Hair Shampoo
 Champô Fortificante e Revitalizante Antiqueda</t>
         </is>
       </c>
-      <c r="C404" s="7" t="inlineStr">
+      <c r="C404" s="3" t="inlineStr">
         <is>
           <t>200 ml</t>
         </is>
       </c>
-      <c r="D404" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="E404" s="7" t="inlineStr">
+      <c r="D404" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="E404" s="3" t="inlineStr">
         <is>
           <t>3000716</t>
         </is>
       </c>
-      <c r="F404" s="7" t="inlineStr">
+      <c r="F404" s="3" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
       </c>
-      <c r="G404" s="7" t="inlineStr">
+      <c r="G404" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/quinine-strengthening-thinning-hair-shampoo-343977.html</t>
         </is>
@@ -22479,40 +22479,40 @@
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="7" t="inlineStr">
-        <is>
-          <t>08/07/2026</t>
-        </is>
-      </c>
-      <c r="B83" s="7" t="inlineStr">
+      <c r="A83" s="5" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
+        </is>
+      </c>
+      <c r="B83" s="5" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C83" s="7" t="inlineStr">
+      <c r="C83" s="5" t="inlineStr">
         <is>
           <t>Intense Eye Make-Up Waterproof Remover
 Desmaquilhante Intenso Olhos Sensíveis
 125 ml</t>
         </is>
       </c>
-      <c r="D83" s="7" t="inlineStr">
+      <c r="D83" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/intense-eye-make-up-waterproof-remover-6661562.html</t>
         </is>
       </c>
-      <c r="E83" s="7" t="inlineStr"/>
-      <c r="F83" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G83" s="7" t="inlineStr">
+      <c r="E83" s="5" t="inlineStr"/>
+      <c r="F83" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G83" s="5" t="inlineStr">
         <is>
           <t>6661562</t>
         </is>
       </c>
-      <c r="H83" s="7" t="inlineStr">
+      <c r="H83" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -22805,40 +22805,40 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="7" t="inlineStr">
-        <is>
-          <t>08/07/2026</t>
-        </is>
-      </c>
-      <c r="B91" s="7" t="inlineStr">
+      <c r="A91" s="3" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
+        </is>
+      </c>
+      <c r="B91" s="3" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C91" s="7" t="inlineStr">
+      <c r="C91" s="3" t="inlineStr">
         <is>
           <t>Milk Cleanser Dry Sensitive Skin
 Leite de Limpeza Desmaquilhante Pele Seca
 200 ml</t>
         </is>
       </c>
-      <c r="D91" s="7" t="inlineStr">
+      <c r="D91" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/milk-cleanser-dry-sensitive-skin-3001085.html</t>
         </is>
       </c>
-      <c r="E91" s="7" t="inlineStr"/>
-      <c r="F91" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G91" s="7" t="inlineStr">
+      <c r="E91" s="3" t="inlineStr"/>
+      <c r="F91" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G91" s="3" t="inlineStr">
         <is>
           <t>3001085</t>
         </is>
       </c>
-      <c r="H91" s="7" t="inlineStr">
+      <c r="H91" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -24332,43 +24332,43 @@
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="7" t="inlineStr">
-        <is>
-          <t>08/07/2026</t>
-        </is>
-      </c>
-      <c r="B129" s="7" t="inlineStr">
+      <c r="A129" s="3" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
+        </is>
+      </c>
+      <c r="B129" s="3" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C129" s="7" t="inlineStr">
+      <c r="C129" s="3" t="inlineStr">
         <is>
           <t>Thermal Spring Water Sensitive Skin
 Água Termal Spray Calmante Instantâneo</t>
         </is>
       </c>
-      <c r="D129" s="7" t="inlineStr">
+      <c r="D129" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/thermal-spring-water-sensitive-skin-431510.html</t>
         </is>
       </c>
-      <c r="E129" s="7" t="inlineStr">
+      <c r="E129" s="3" t="inlineStr">
         <is>
           <t>50 ml</t>
         </is>
       </c>
-      <c r="F129" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G129" s="7" t="inlineStr">
+      <c r="F129" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G129" s="3" t="inlineStr">
         <is>
           <t>3000998</t>
         </is>
       </c>
-      <c r="H129" s="7" t="inlineStr">
+      <c r="H129" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -25630,40 +25630,40 @@
       </c>
     </row>
     <row r="161">
-      <c r="A161" s="7" t="inlineStr">
-        <is>
-          <t>08/07/2026</t>
-        </is>
-      </c>
-      <c r="B161" s="7" t="inlineStr">
+      <c r="A161" s="5" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
+        </is>
+      </c>
+      <c r="B161" s="5" t="inlineStr">
         <is>
           <t>Avène</t>
         </is>
       </c>
-      <c r="C161" s="7" t="inlineStr">
+      <c r="C161" s="5" t="inlineStr">
         <is>
           <t>Xeracalm NUTRITION Shower Cream
 Creme Duche Sem Sabão Pele Muito Seca
 500 ml</t>
         </is>
       </c>
-      <c r="D161" s="7" t="inlineStr">
+      <c r="D161" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/xeracalm-nutrition-shower-cream-7816797.html</t>
         </is>
       </c>
-      <c r="E161" s="7" t="inlineStr"/>
-      <c r="F161" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G161" s="7" t="inlineStr">
+      <c r="E161" s="5" t="inlineStr"/>
+      <c r="F161" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G161" s="5" t="inlineStr">
         <is>
           <t>7816797</t>
         </is>
       </c>
-      <c r="H161" s="7" t="inlineStr">
+      <c r="H161" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -29086,40 +29086,40 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t>08/07/2026</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>Centaury Anti-Yellowing Gray, Blond Shampoo
 Champô Centáurea BIO Neutraliza Tons Amarelos
 400 ml</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/centaury-anti-yellowing-gray-blond-shampoo-6863851.html</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr"/>
-      <c r="F10" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G10" s="7" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr"/>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>6863851</t>
         </is>
       </c>
-      <c r="H10" s="7" t="inlineStr">
+      <c r="H10" s="3" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
@@ -29452,40 +29452,40 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="7" t="inlineStr">
-        <is>
-          <t>08/07/2026</t>
-        </is>
-      </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="C19" s="7" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr">
         <is>
           <t>Crème Solaire Sublime SPF 50+
 Protetor Solar de Rosto Antienvelhecimento
 50 ml</t>
         </is>
       </c>
-      <c r="D19" s="7" t="inlineStr">
+      <c r="D19" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/creme-solaire-sublime-spf-50-7129219.html</t>
         </is>
       </c>
-      <c r="E19" s="7" t="inlineStr"/>
-      <c r="F19" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G19" s="7" t="inlineStr">
+      <c r="E19" s="3" t="inlineStr"/>
+      <c r="F19" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
         <is>
           <t>7129219</t>
         </is>
       </c>
-      <c r="H19" s="7" t="inlineStr">
+      <c r="H19" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -29852,40 +29852,40 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="7" t="inlineStr">
-        <is>
-          <t>08/07/2026</t>
-        </is>
-      </c>
-      <c r="B29" s="7" t="inlineStr">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="C29" s="7" t="inlineStr">
+      <c r="C29" s="3" t="inlineStr">
         <is>
           <t>Cupuaçu Reparing Very Dry Hair Shampoo
 Champô Cupuaçu BIO Repara Cabelo Muito Seco
 400 ml</t>
         </is>
       </c>
-      <c r="D29" s="7" t="inlineStr">
+      <c r="D29" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/cupuacu-reparing-very-dry-hair-shampoo-343983.html</t>
         </is>
       </c>
-      <c r="E29" s="7" t="inlineStr"/>
-      <c r="F29" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G29" s="7" t="inlineStr">
+      <c r="E29" s="3" t="inlineStr"/>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
         <is>
           <t>7104602</t>
         </is>
       </c>
-      <c r="H29" s="7" t="inlineStr">
+      <c r="H29" s="3" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
@@ -30873,43 +30873,43 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="7" t="inlineStr">
-        <is>
-          <t>08/07/2026</t>
-        </is>
-      </c>
-      <c r="B54" s="7" t="inlineStr">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="C54" s="7" t="inlineStr">
+      <c r="C54" s="3" t="inlineStr">
         <is>
           <t>Mango Nourishing Shampoo
 Champô Manga Nutritivo para Cabelo Seco</t>
         </is>
       </c>
-      <c r="D54" s="7" t="inlineStr">
+      <c r="D54" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/mango-nourishing-shampoo-344278.html</t>
         </is>
       </c>
-      <c r="E54" s="7" t="inlineStr">
+      <c r="E54" s="3" t="inlineStr">
         <is>
           <t>100 ml</t>
         </is>
       </c>
-      <c r="F54" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G54" s="7" t="inlineStr">
+      <c r="F54" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G54" s="3" t="inlineStr">
         <is>
           <t>6128309</t>
         </is>
       </c>
-      <c r="H54" s="7" t="inlineStr">
+      <c r="H54" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -31918,43 +31918,43 @@
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="7" t="inlineStr">
-        <is>
-          <t>08/07/2026</t>
-        </is>
-      </c>
-      <c r="B79" s="7" t="inlineStr">
+      <c r="A79" s="5" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
+        </is>
+      </c>
+      <c r="B79" s="5" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="C79" s="7" t="inlineStr">
+      <c r="C79" s="5" t="inlineStr">
         <is>
           <t>Prickly Pear 72h Hydration &amp; Shine Shampoo
 Champô Figo da Índia Hidratante Cabelo Baço</t>
         </is>
       </c>
-      <c r="D79" s="7" t="inlineStr">
+      <c r="D79" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/prickly-pear-72h-hydration-and-shine-shampoo-355576.html</t>
         </is>
       </c>
-      <c r="E79" s="7" t="inlineStr">
+      <c r="E79" s="5" t="inlineStr">
         <is>
           <t>400 ml</t>
         </is>
       </c>
-      <c r="F79" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G79" s="7" t="inlineStr">
+      <c r="F79" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G79" s="5" t="inlineStr">
         <is>
           <t>8067439</t>
         </is>
       </c>
-      <c r="H79" s="7" t="inlineStr">
+      <c r="H79" s="5" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
@@ -32204,43 +32204,43 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="7" t="inlineStr">
-        <is>
-          <t>08/07/2026</t>
-        </is>
-      </c>
-      <c r="B86" s="7" t="inlineStr">
+      <c r="A86" s="5" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
+        </is>
+      </c>
+      <c r="B86" s="5" t="inlineStr">
         <is>
           <t>Klorane</t>
         </is>
       </c>
-      <c r="C86" s="7" t="inlineStr">
+      <c r="C86" s="5" t="inlineStr">
         <is>
           <t>Quinine Strengthening Thinning Hair Shampoo
 Champô Fortificante e Revitalizante Antiqueda</t>
         </is>
       </c>
-      <c r="D86" s="7" t="inlineStr">
+      <c r="D86" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/quinine-strengthening-thinning-hair-shampoo-343977.html</t>
         </is>
       </c>
-      <c r="E86" s="7" t="inlineStr">
+      <c r="E86" s="5" t="inlineStr">
         <is>
           <t>200 ml</t>
         </is>
       </c>
-      <c r="F86" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G86" s="7" t="inlineStr">
+      <c r="F86" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G86" s="5" t="inlineStr">
         <is>
           <t>3000716</t>
         </is>
       </c>
-      <c r="H86" s="7" t="inlineStr">
+      <c r="H86" s="5" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
@@ -34373,40 +34373,40 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="7" t="inlineStr">
-        <is>
-          <t>08/07/2026</t>
-        </is>
-      </c>
-      <c r="B47" s="7" t="inlineStr">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C47" s="7" t="inlineStr">
+      <c r="C47" s="3" t="inlineStr">
         <is>
           <t>Style Texture Spray Volume &amp; Hold
 Spray Cabelo Texturizante Volumizador da Raiz
 200 ml</t>
         </is>
       </c>
-      <c r="D47" s="7" t="inlineStr">
+      <c r="D47" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/style-texture-spray-volume-and-hold-7447303.html</t>
         </is>
       </c>
-      <c r="E47" s="7" t="inlineStr"/>
-      <c r="F47" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G47" s="7" t="inlineStr">
+      <c r="E47" s="3" t="inlineStr"/>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G47" s="3" t="inlineStr">
         <is>
           <t>7447303</t>
         </is>
       </c>
-      <c r="H47" s="7" t="inlineStr">
+      <c r="H47" s="3" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
@@ -35219,40 +35219,40 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="7" t="inlineStr">
-        <is>
-          <t>08/07/2026</t>
-        </is>
-      </c>
-      <c r="B68" s="7" t="inlineStr">
+      <c r="A68" s="3" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
         <is>
           <t>René Furterer</t>
         </is>
       </c>
-      <c r="C68" s="7" t="inlineStr">
+      <c r="C68" s="3" t="inlineStr">
         <is>
           <t>Triphasic Reactional Cuidado 2 em 1 Antiqueda
 Ampolas para Queda de Cabelo Reativa
 12 un</t>
         </is>
       </c>
-      <c r="D68" s="7" t="inlineStr">
+      <c r="D68" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/triphasic-reactional-cuidado-2-em-1-antiqueda-6856572.html</t>
         </is>
       </c>
-      <c r="E68" s="7" t="inlineStr"/>
-      <c r="F68" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G68" s="7" t="inlineStr">
+      <c r="E68" s="3" t="inlineStr"/>
+      <c r="F68" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G68" s="3" t="inlineStr">
         <is>
           <t>6856572</t>
         </is>
       </c>
-      <c r="H68" s="7" t="inlineStr">
+      <c r="H68" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -36730,43 +36730,43 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="7" t="inlineStr">
-        <is>
-          <t>08/07/2026</t>
-        </is>
-      </c>
-      <c r="B31" s="7" t="inlineStr">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
         <is>
           <t>A-Derma</t>
         </is>
       </c>
-      <c r="C31" s="7" t="inlineStr">
+      <c r="C31" s="5" t="inlineStr">
         <is>
           <t>Exomega Control Emolient Shower Oil
 Óleo Banho Calmante Comichão da Pele Atópica</t>
         </is>
       </c>
-      <c r="D31" s="7" t="inlineStr">
+      <c r="D31" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/exomega-control-emolient-shower-oil-452817.html</t>
         </is>
       </c>
-      <c r="E31" s="7" t="inlineStr">
+      <c r="E31" s="5" t="inlineStr">
         <is>
           <t>1000 ml</t>
         </is>
       </c>
-      <c r="F31" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G31" s="7" t="inlineStr">
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G31" s="5" t="inlineStr">
         <is>
           <t>8605683</t>
         </is>
       </c>
-      <c r="H31" s="7" t="inlineStr">
+      <c r="H31" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -38003,40 +38003,40 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="7" t="inlineStr">
-        <is>
-          <t>08/07/2026</t>
-        </is>
-      </c>
-      <c r="B62" s="7" t="inlineStr">
+      <c r="A62" s="3" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
         <is>
           <t>A-Derma</t>
         </is>
       </c>
-      <c r="C62" s="7" t="inlineStr">
+      <c r="C62" s="3" t="inlineStr">
         <is>
           <t>Soothing Dermatololical Bar
 Sabonete Dermatológico para a Pele Sensível
 100gr</t>
         </is>
       </c>
-      <c r="D62" s="7" t="inlineStr">
+      <c r="D62" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/soothing-dermatololical-bar-3026152.html</t>
         </is>
       </c>
-      <c r="E62" s="7" t="inlineStr"/>
-      <c r="F62" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G62" s="7" t="inlineStr">
+      <c r="E62" s="3" t="inlineStr"/>
+      <c r="F62" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G62" s="3" t="inlineStr">
         <is>
           <t>3026152</t>
         </is>
       </c>
-      <c r="H62" s="7" t="inlineStr">
+      <c r="H62" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -38436,17 +38436,17 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t>08/07/2026</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
         <is>
           <t>Oral Care</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>Eludril
 Daily Mouthwash Protect
@@ -38454,63 +38454,63 @@
 500 ml x 2</t>
         </is>
       </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/daily-mouthwash-protect-8437650.html</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr"/>
-      <c r="F9" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G9" s="7" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr"/>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
         <is>
           <t>8437650</t>
         </is>
       </c>
-      <c r="H9" s="7" t="inlineStr">
+      <c r="H9" s="5" t="inlineStr">
         <is>
           <t>Sem desconto</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t>08/07/2026</t>
-        </is>
-      </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>Oral Care</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t>Elgydium
 Dentífrico Baby Bio
 30 ml</t>
         </is>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/dentifrico-baby-bio-7697224.html</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr"/>
-      <c r="F10" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G10" s="7" t="inlineStr">
+      <c r="E10" s="3" t="inlineStr"/>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>7697224</t>
         </is>
       </c>
-      <c r="H10" s="7" t="inlineStr">
+      <c r="H10" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -38677,40 +38677,40 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="inlineStr">
-        <is>
-          <t>08/07/2026</t>
-        </is>
-      </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>Oral Care</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>Elgydium
 Elgydium Fix Fixação Forte
 45 g</t>
         </is>
       </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/elgydium-fix-fixacao-forte-7434256.html</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr"/>
-      <c r="F15" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G15" s="7" t="inlineStr">
+      <c r="E15" s="5" t="inlineStr"/>
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
         <is>
           <t>7434256</t>
         </is>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="H15" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -40363,40 +40363,40 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="7" t="inlineStr">
-        <is>
-          <t>08/07/2026</t>
-        </is>
-      </c>
-      <c r="B57" s="7" t="inlineStr">
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
         <is>
           <t>Oral Care</t>
         </is>
       </c>
-      <c r="C57" s="7" t="inlineStr">
+      <c r="C57" s="5" t="inlineStr">
         <is>
           <t>Elgydium
 Escovilhões Clinic Mono Pretos
 4 un</t>
         </is>
       </c>
-      <c r="D57" s="7" t="inlineStr">
+      <c r="D57" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/escovilhoes-clinic-mono-pretos-6937302.html</t>
         </is>
       </c>
-      <c r="E57" s="7" t="inlineStr"/>
-      <c r="F57" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G57" s="7" t="inlineStr">
+      <c r="E57" s="5" t="inlineStr"/>
+      <c r="F57" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G57" s="5" t="inlineStr">
         <is>
           <t>6937302</t>
         </is>
       </c>
-      <c r="H57" s="7" t="inlineStr">
+      <c r="H57" s="5" t="inlineStr">
         <is>
           <t>25%</t>
         </is>
@@ -41287,40 +41287,40 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="7" t="inlineStr">
-        <is>
-          <t>08/07/2026</t>
-        </is>
-      </c>
-      <c r="B80" s="7" t="inlineStr">
+      <c r="A80" s="3" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
+        </is>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
         <is>
           <t>Oral Care</t>
         </is>
       </c>
-      <c r="C80" s="7" t="inlineStr">
+      <c r="C80" s="3" t="inlineStr">
         <is>
           <t>Arthrodont
 Pasta de Dentes Gengivas Irritadas
 75 ml</t>
         </is>
       </c>
-      <c r="D80" s="7" t="inlineStr">
+      <c r="D80" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/pasta-de-dentes-gengivas-irritadas-3045806.html</t>
         </is>
       </c>
-      <c r="E80" s="7" t="inlineStr"/>
-      <c r="F80" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G80" s="7" t="inlineStr">
+      <c r="E80" s="3" t="inlineStr"/>
+      <c r="F80" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G80" s="3" t="inlineStr">
         <is>
           <t>3045806</t>
         </is>
       </c>
-      <c r="H80" s="7" t="inlineStr">
+      <c r="H80" s="3" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
@@ -41814,17 +41814,17 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="7" t="inlineStr">
-        <is>
-          <t>08/07/2026</t>
-        </is>
-      </c>
-      <c r="B93" s="7" t="inlineStr">
+      <c r="A93" s="5" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
+        </is>
+      </c>
+      <c r="B93" s="5" t="inlineStr">
         <is>
           <t>Oral Care</t>
         </is>
       </c>
-      <c r="C93" s="7" t="inlineStr">
+      <c r="C93" s="5" t="inlineStr">
         <is>
           <t>Eludril
 Sensitive Colutório Uso Diário
@@ -41832,23 +41832,23 @@
 500 ml</t>
         </is>
       </c>
-      <c r="D93" s="7" t="inlineStr">
+      <c r="D93" s="5" t="inlineStr">
         <is>
           <t>https://wells.pt/sensitive-colutorio-uso-diario-7407495.html</t>
         </is>
       </c>
-      <c r="E93" s="7" t="inlineStr"/>
-      <c r="F93" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G93" s="7" t="inlineStr">
+      <c r="E93" s="5" t="inlineStr"/>
+      <c r="F93" s="6" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G93" s="5" t="inlineStr">
         <is>
           <t>7407495</t>
         </is>
       </c>
-      <c r="H93" s="7" t="inlineStr">
+      <c r="H93" s="5" t="inlineStr">
         <is>
           <t>Sem desconto</t>
         </is>
@@ -41936,40 +41936,40 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="7" t="inlineStr">
-        <is>
-          <t>08/07/2026</t>
-        </is>
-      </c>
-      <c r="B96" s="7" t="inlineStr">
+      <c r="A96" s="3" t="inlineStr">
+        <is>
+          <t>08/07/2026</t>
+        </is>
+      </c>
+      <c r="B96" s="3" t="inlineStr">
         <is>
           <t>Oral Care</t>
         </is>
       </c>
-      <c r="C96" s="7" t="inlineStr">
+      <c r="C96" s="3" t="inlineStr">
         <is>
           <t>Elgydium
 Spray Xeroleave Boca Seca
 70 ml</t>
         </is>
       </c>
-      <c r="D96" s="7" t="inlineStr">
+      <c r="D96" s="3" t="inlineStr">
         <is>
           <t>https://wells.pt/spray-xeroleave-boca-seca-6259717.html</t>
         </is>
       </c>
-      <c r="E96" s="7" t="inlineStr"/>
-      <c r="F96" s="8" t="inlineStr">
-        <is>
-          <t>Out of Stock</t>
-        </is>
-      </c>
-      <c r="G96" s="7" t="inlineStr">
+      <c r="E96" s="3" t="inlineStr"/>
+      <c r="F96" s="4" t="inlineStr">
+        <is>
+          <t>In Stock</t>
+        </is>
+      </c>
+      <c r="G96" s="3" t="inlineStr">
         <is>
           <t>6259717</t>
         </is>
       </c>
-      <c r="H96" s="7" t="inlineStr">
+      <c r="H96" s="3" t="inlineStr">
         <is>
           <t>25%</t>
         </is>

</xml_diff>